<commit_message>
Clarify tariff source usage
</commit_message>
<xml_diff>
--- a/Excel/Line-Energy-Solar-Calculator-v0.13.xlsx
+++ b/Excel/Line-Energy-Solar-Calculator-v0.13.xlsx
@@ -4449,7 +4449,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Starter values only; verify current retail tariff and microgeneration purchase price for exact supplier/date.</t>
+          <t>Retail tariff: verify with regional supplier/regulator. Export price: verify through ATS market-price data used for microgeneration surplus purchase.</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Starter values only; verify current retail tariff and microgeneration purchase price for exact supplier/date.</t>
+          <t>Retail tariff: verify with regional supplier/regulator. Export price: verify through ATS market-price data used for microgeneration surplus purchase.</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Starter values only; verify current retail tariff and microgeneration purchase price for exact supplier/date.</t>
+          <t>Retail tariff: verify with regional supplier/regulator. Export price: verify through ATS market-price data used for microgeneration surplus purchase.</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Starter values only; verify current retail tariff and microgeneration purchase price for exact supplier/date.</t>
+          <t>Retail tariff: verify with regional supplier/regulator. Export price: verify through ATS market-price data used for microgeneration surplus purchase.</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Starter values only; verify current retail tariff and microgeneration purchase price for exact supplier/date.</t>
+          <t>Retail tariff: verify with regional supplier/regulator. Export price: verify through ATS market-price data used for microgeneration surplus purchase.</t>
         </is>
       </c>
     </row>

</xml_diff>